<commit_message>
Simple Flow V2: friendlier multi-tab question workbook for Milos
Rebuilt the PO question sheet as an attractive 6-tab workbook (Start here /
one tab per question with a yellow answer box + notes / All-3-at-a-glance /
QA-internal references) and uploaded it to the PO's Drive; it opens and edits
directly in Google Sheets with all tabs intact. PO questions super-simplified
to plain one-line wording with tick-box options; all case-ids/spec anchors
kept on the QA-internal tab only. Docs updated with the new link.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QvLHRX1rY5c7HuyoMWVGpU
</commit_message>
<xml_diff>
--- a/build/simple-flow-v2/source-verify-2026-09-08/Simple Flow V2 - Questions for Milos Vasic - 2026-09-08.xlsx
+++ b/build/simple-flow-v2/source-verify-2026-09-08/Simple Flow V2 - Questions for Milos Vasic - 2026-09-08.xlsx
@@ -7,8 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Questions for the PO" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="QA internal - not for the PO" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="👋 Start here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="1️⃣ Question 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2️⃣ Question 2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="3️⃣ Question 3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="⚡ All 3 at a glance" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="🔒 QA internal (ignore)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,13 +32,44 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="13"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -43,11 +78,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDDDDD"/>
+        <fgColor rgb="001F3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F0F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E5E8C"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -55,18 +115,81 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,148 +555,99 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Simple Flow V2 - Questions for Milos Vasic</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>Simple Flow V2 — a few quick questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Three quick questions came up while we checked the Simple Flow V2 tests against the latest notes (8 September 2026). Please tick one option per row, and add a note if you like. Nothing technical is needed to answer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Hi Milos — thanks for taking a look. This should take about two minutes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="46" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Topic</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>What happens now</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>The question</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Options</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Your answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Changing several settings at the same time</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>When several of these settings are changed together, the 'approval' one is applied first. But changing 'approval' never changes any work that already exists.</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Since it never changes existing work, does applying 'approval' first matter at all - or does it simply mean that work still waiting for approval is left out when the other settings are applied?</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>A) It simply means work still waiting for approval is left out - nothing else to check. B) It does something else we should check (please describe).</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>The 'Select all' box on the receive list</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>The receive list shows about thirty at a time and loads more as you scroll down.</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>'Select all' ticks only the ones already on screen, not the ones further down. Is that okay for now?</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>A) Yes, that is fine for now. B) No - it should tick every one; please raise it as a problem to fix.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Very large changes</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>A small change happens straight away on screen. A very large one runs quietly in the background, and shows advice to make it after working hours.</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>How many affected jobs count as 'too large to do on screen', and how many should trigger the 'do it after hours' advice? (An engineer may need to answer.)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>A) Here are the two numbers. B) Not decided yet - for now, just check that the wait affects the admin who made the change and no one else.</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>What is this?</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>While preparing the tests for Simple Flow V2, three small things weren't clear from the written notes. Your answer settles each one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>How to answer</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Open the tab for each question (Question 1, 2, 3 along the bottom). Read the short description, then type A or B in the yellow ‘Your answer’ box. Add a note if you want — totally optional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>In a hurry?</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Use the ‘⚡ All 3 at a glance’ tab to answer all three in one place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>No jargon</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Everything is in plain language — you don't need any technical detail to answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Thank you 🙏</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>That's it. Your answers let us finish the tests correctly. Much appreciated!</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -584,111 +658,554 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="76" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>This sheet is for us. It is the traceability the PO does not need to read.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Question #</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Changing several settings at once</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Please read the two short boxes, then type A or B in the yellow box.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>What happens now</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>When an admin changes several of these settings together, the ‘approval’ setting is applied first. But changing ‘approval’ never changes any work that already exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>The question</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Does applying ‘approval’ first actually change anything — or does it simply mean that work still waiting for approval is skipped when the other settings are applied?</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Option A</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>A — It simply means work waiting for approval is skipped. Nothing else to check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Option B</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>B — Applying it first does something else we should check. (Please tell us what, in Notes.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>👉 Your answer</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>(type A or B here)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11" ht="24" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B10:D11"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>The ‘Select all’ box on the receive list</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Please read the two short boxes, then type A or B in the yellow box.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>What happens now</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>The receive list shows about thirty rows at a time and loads more as you scroll down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>The question</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>When you press ‘Select all’, it ticks only the rows already on screen (about thirty) — not the ones further down. Is that okay for now?</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Option A</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>A — Yes, that's fine for now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Option B</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>B — No, ‘Select all’ should tick every row. Please raise it as a problem to fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>👉 Your answer</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>(type A or B here)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11" ht="24" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B10:D11"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Very large changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Please read the two short boxes, then type A or B in the yellow box.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>What happens now</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>A small change happens straight away on screen. A very large one runs quietly in the background, and the screen shows advice to make it after working hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>The question</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>How many affected jobs count as ‘too large to do on screen’, and how many should trigger the ‘do it after hours’ advice? (An engineer may need to give the numbers.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Option A</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>A — Here are the two numbers: ____ and ____ (type them in Notes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Option B</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>B — Not decided yet — for now just check the wait affects only the admin who made the change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>👉 Your answer</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>(type A or B here)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11" ht="24" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B10:D11"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>All three questions — answer here if you prefer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Type A or B in each yellow box. Full detail is on the numbered tabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>The question in one line</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Your answer (A/B)</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="56" customHeight="1">
+      <c r="A5" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>When several settings change at once, does ‘approval first’ matter, or does it just skip work still awaiting approval?</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr"/>
+      <c r="D5" s="13" t="inlineStr"/>
+    </row>
+    <row r="6" ht="56" customHeight="1">
+      <c r="A6" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Is it okay that ‘Select all’ ticks only the ~30 rows on screen, not the ones further down?</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr"/>
+      <c r="D6" s="13" t="inlineStr"/>
+    </row>
+    <row r="7" ht="56" customHeight="1">
+      <c r="A7" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>What are the two size limits for ‘runs in the background’ and ‘do it after hours’ advice?</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr"/>
+      <c r="D7" s="13" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>QA internal — references (not for the PO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>For us. The traceability the PO does not need to read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Q#</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Cases it decides</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Why it is a question and not a defect</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Why it is a question, not a defect</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="70" customHeight="1">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>C44554 - https://shopview.testrail.io/index.php?/cases/view/44554</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>C44554 — https://shopview.testrail.io/index.php?/cases/view/44554</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Epic SV-8683 / Story SV-9248 (Story 2) / spec 771391574 (rev 8 Sep 2026), Story 2 Requirements</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Spec states both 'approval applied first, then ordering, then picking' AND 'turning approval on or off changes no existing line'. If approval never sweeps existing lines the precedence is a no-op on existing data. C44554 item 5 tests only the exclusion of not-yet-approved parts from the ordering/picking sweeps; the precedence itself is left unwritten pending Milos. A genuine spec ambiguity, not a defect.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>Spec says both ‘approval applied first, then ordering, then picking’ AND ‘turning approval on/off changes no existing line’. If approval never sweeps, precedence is a no-op on existing data. C44554 item 5 tests only exclusion of not-yet-approved parts; precedence left unwritten pending Milos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>C53488 - https://shopview.testrail.io/index.php?/cases/view/53488</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Epic SV-8683 / Story SV-9260 (Story 14) / spec 771391574 (rev 8 Sep 2026), Story 14 'The receive page and PO bulk receive'</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Spec records paged 'Select all' (loads one page, ~30 rows) as EXPECTED behaviour, not a defect, resolving when pagination is replaced - which is outside this release. Confirming keeps C53488 a Pass rather than a raised deviation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>C53488 — https://shopview.testrail.io/index.php?/cases/view/53488</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>Epic SV-8683 / Story SV-9260 (Story 14) / spec 771391574 (rev 8 Sep 2026), Story 14 receive page &amp; PO bulk receive</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Spec records paged Select-all (one page, ~30 rows) as EXPECTED, resolving when pagination is replaced — outside this release. Confirming keeps C53488 a Pass, not a raised deviation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>C44559 - https://shopview.testrail.io/index.php?/cases/view/44559</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Epic SV-8683 / Story SV-9250 (Story 4) / spec 771391574 (rev 8 Sep 2026), Story 4 'Applying at scale'</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>The two volume thresholds (in-request vs background application; and the off-hours advisory trigger) are 'agreed with engineering', not stated in the spec. The admin-only-blocking behaviour is testable now (C44559); the two boundaries need concrete numbers. Engineering answer, relayed via Milos.</t>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>C44559 — https://shopview.testrail.io/index.php?/cases/view/44559</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>Epic SV-8683 / Story SV-9250 (Story 4) / spec 771391574 (rev 8 Sep 2026), Story 4 Applying at scale</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Two volume thresholds (in-request vs background; off-hours advisory) are ‘agreed with engineering’, not stated. Admin-only-blocking is testable now (C44559); the two boundaries need concrete numbers.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>